<commit_message>
Refactor Groups POM and update tests
Major refactor of GroupsAddGroups POM: reorganized fields and methods, added clearer sections (navigation, add group, add/remove device, delete), scoped/fixed locators, improved waits/notification handling, and added utility methods (deleteAllGroups, isGroupCreated, isDeviceAdded/Removed). Added Eclipse encoding prefs (.settings/org.eclipse.core.resources.prefs). Updated baseTest to use instance driver, added @AfterClass tearDown to reliably quit browser, and kept DataProvider. Updated groupPageTest: split and restructured tests (login, addSingleGroup, deleteGroups, device add/remove flows), improved assertions and test dependencies. Test resources and generated test reports/targets updated (data.xlsx, pom.properties and test-output files) as part of running the suite.
</commit_message>
<xml_diff>
--- a/src/test/resources/data.xlsx
+++ b/src/test/resources/data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23415" windowHeight="7620" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23415" windowHeight="7620"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
@@ -21530,41 +21530,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="B2" r:id="rId2"/>
-    <hyperlink ref="A3" r:id="rId3"/>
-    <hyperlink ref="B3" r:id="rId4"/>
-    <hyperlink ref="B1" r:id="rId5"/>
-    <hyperlink ref="A1" r:id="rId6"/>
+    <hyperlink ref="A1" r:id="rId1"/>
+    <hyperlink ref="B1" r:id="rId2"/>
+    <hyperlink ref="A2" r:id="rId3"/>
+    <hyperlink ref="B2" r:id="rId4"/>
+    <hyperlink ref="B3" r:id="rId5"/>
+    <hyperlink ref="A3" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>